<commit_message>
Atualização automática das bases ECODATA
</commit_message>
<xml_diff>
--- a/data/final/bcb_sgs/base_bcb_sgs_mensal_larga.xlsx
+++ b/data/final/bcb_sgs/base_bcb_sgs_mensal_larga.xlsx
@@ -7183,11 +7183,15 @@
       <c r="D61" t="n">
         <v>0.053028</v>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>0.16</v>
+      </c>
       <c r="F61" t="n">
         <v>-0.5</v>
       </c>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="n">
+        <v>0.14</v>
+      </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="n">
@@ -7220,11 +7224,15 @@
       <c r="AA61" t="n">
         <v>-0.964334</v>
       </c>
-      <c r="AB61" t="inlineStr"/>
+      <c r="AB61" t="n">
+        <v>4.641328</v>
+      </c>
       <c r="AC61" t="n">
         <v>3.177699</v>
       </c>
-      <c r="AD61" t="inlineStr"/>
+      <c r="AD61" t="n">
+        <v>4.327084</v>
+      </c>
       <c r="AE61" t="n">
         <v>-0.25</v>
       </c>
@@ -7258,10 +7266,10 @@
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="n">
-        <v>5.1329</v>
+        <v>5.1088</v>
       </c>
       <c r="K62" t="n">
-        <v>5.1323</v>
+        <v>5.1082</v>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
@@ -7274,10 +7282,10 @@
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="n">
-        <v>-0.844183</v>
+        <v>-1.30974</v>
       </c>
       <c r="W62" t="n">
-        <v>-0.8442809999999999</v>
+        <v>-1.309892</v>
       </c>
       <c r="X62" t="inlineStr"/>
       <c r="Y62" t="inlineStr"/>

</xml_diff>